<commit_message>
#52 LCSC And PCBWay BOM added.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Espark_BOM.xlsx
+++ b/Deliverables/BOM/Espark_BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\JohnWollam-LCDProject\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{014C0970-D35D-495B-827E-575320382BA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A71E665-A050-4A05-A973-21CA348C056A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1602,6 +1602,77 @@
     <xf numFmtId="166" fontId="17" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1630,77 +1701,6 @@
     <xf numFmtId="0" fontId="28" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2085,15 +2085,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-      <c r="P1" s="101"/>
-      <c r="Q1" s="101"/>
-      <c r="R1" s="101"/>
-      <c r="S1" s="102"/>
+      <c r="K1" s="128"/>
+      <c r="L1" s="128"/>
+      <c r="M1" s="128"/>
+      <c r="N1" s="128"/>
+      <c r="O1" s="128"/>
+      <c r="P1" s="128"/>
+      <c r="Q1" s="128"/>
+      <c r="R1" s="128"/>
+      <c r="S1" s="129"/>
     </row>
     <row r="2" spans="1:27" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2118,27 +2118,27 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
-      <c r="S2" s="104"/>
-      <c r="T2" s="104"/>
-      <c r="U2" s="104"/>
-      <c r="V2" s="104"/>
-      <c r="W2" s="105"/>
+      <c r="S2" s="131"/>
+      <c r="T2" s="131"/>
+      <c r="U2" s="131"/>
+      <c r="V2" s="131"/>
+      <c r="W2" s="132"/>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="17"/>
-      <c r="C3" s="110"/>
-      <c r="D3" s="111" t="s">
+      <c r="C3" s="101"/>
+      <c r="D3" s="102" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="111"/>
-      <c r="F3" s="112" t="s">
+      <c r="E3" s="102"/>
+      <c r="F3" s="103" t="s">
         <v>224</v>
       </c>
-      <c r="G3" s="111"/>
-      <c r="H3" s="113"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="113"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="104"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="104"/>
       <c r="K3" s="39"/>
       <c r="L3" s="39"/>
       <c r="M3" s="39"/>
@@ -2151,16 +2151,16 @@
       <c r="T3" s="40"/>
       <c r="U3" s="40"/>
       <c r="V3" s="40"/>
-      <c r="W3" s="103"/>
+      <c r="W3" s="130"/>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="17"/>
-      <c r="C4" s="110"/>
-      <c r="D4" s="111" t="s">
+      <c r="C4" s="101"/>
+      <c r="D4" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="111"/>
+      <c r="E4" s="102"/>
       <c r="F4" s="33" t="s">
         <v>224</v>
       </c>
@@ -2180,16 +2180,16 @@
       <c r="T4" s="36"/>
       <c r="U4" s="36"/>
       <c r="V4" s="36"/>
-      <c r="W4" s="103"/>
+      <c r="W4" s="130"/>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="17"/>
-      <c r="C5" s="110"/>
-      <c r="D5" s="111" t="s">
+      <c r="C5" s="101"/>
+      <c r="D5" s="102" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="111"/>
+      <c r="E5" s="102"/>
       <c r="F5" s="34" t="s">
         <v>5</v>
       </c>
@@ -2209,7 +2209,7 @@
       <c r="T5" s="37"/>
       <c r="U5" s="37"/>
       <c r="V5" s="37"/>
-      <c r="W5" s="103"/>
+      <c r="W5" s="130"/>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2234,57 +2234,57 @@
       <c r="T6" s="37"/>
       <c r="U6" s="37"/>
       <c r="V6" s="37"/>
-      <c r="W6" s="103"/>
+      <c r="W6" s="130"/>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="19"/>
-      <c r="C7" s="114"/>
-      <c r="D7" s="115"/>
-      <c r="E7" s="115"/>
+      <c r="C7" s="105"/>
+      <c r="D7" s="106"/>
+      <c r="E7" s="106"/>
       <c r="F7" s="14"/>
-      <c r="G7" s="115"/>
-      <c r="H7" s="116"/>
-      <c r="I7" s="115"/>
-      <c r="J7" s="116"/>
-      <c r="K7" s="116"/>
-      <c r="L7" s="116"/>
-      <c r="M7" s="116"/>
-      <c r="N7" s="116"/>
-      <c r="O7" s="116"/>
-      <c r="P7" s="116"/>
-      <c r="Q7" s="116"/>
-      <c r="R7" s="117"/>
-      <c r="S7" s="117"/>
-      <c r="T7" s="117"/>
-      <c r="U7" s="117"/>
-      <c r="V7" s="117"/>
-      <c r="W7" s="103"/>
+      <c r="G7" s="106"/>
+      <c r="H7" s="107"/>
+      <c r="I7" s="106"/>
+      <c r="J7" s="107"/>
+      <c r="K7" s="107"/>
+      <c r="L7" s="107"/>
+      <c r="M7" s="107"/>
+      <c r="N7" s="107"/>
+      <c r="O7" s="107"/>
+      <c r="P7" s="107"/>
+      <c r="Q7" s="107"/>
+      <c r="R7" s="108"/>
+      <c r="S7" s="108"/>
+      <c r="T7" s="108"/>
+      <c r="U7" s="108"/>
+      <c r="V7" s="108"/>
+      <c r="W7" s="130"/>
     </row>
     <row r="8" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="22"/>
-      <c r="C8" s="118"/>
-      <c r="D8" s="119"/>
-      <c r="E8" s="119"/>
-      <c r="F8" s="120"/>
-      <c r="G8" s="115"/>
-      <c r="H8" s="116"/>
-      <c r="I8" s="115"/>
-      <c r="J8" s="116"/>
-      <c r="K8" s="116"/>
-      <c r="L8" s="116"/>
-      <c r="M8" s="116"/>
-      <c r="N8" s="116"/>
-      <c r="O8" s="116"/>
-      <c r="P8" s="116"/>
-      <c r="Q8" s="116"/>
+      <c r="C8" s="109"/>
+      <c r="D8" s="110"/>
+      <c r="E8" s="110"/>
+      <c r="F8" s="111"/>
+      <c r="G8" s="106"/>
+      <c r="H8" s="107"/>
+      <c r="I8" s="106"/>
+      <c r="J8" s="107"/>
+      <c r="K8" s="107"/>
+      <c r="L8" s="107"/>
+      <c r="M8" s="107"/>
+      <c r="N8" s="107"/>
+      <c r="O8" s="107"/>
+      <c r="P8" s="107"/>
+      <c r="Q8" s="107"/>
       <c r="R8" s="35"/>
       <c r="S8" s="35"/>
       <c r="T8" s="35"/>
       <c r="U8" s="35"/>
       <c r="V8" s="35"/>
-      <c r="W8" s="103"/>
+      <c r="W8" s="130"/>
     </row>
     <row r="9" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2357,11 +2357,11 @@
     </row>
     <row r="10" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="135">
+      <c r="B10" s="126">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="129" t="s">
+      <c r="C10" s="120" t="s">
         <v>162</v>
       </c>
       <c r="D10" s="90" t="s">
@@ -2423,18 +2423,18 @@
         <v>0.57999999999999996</v>
       </c>
       <c r="V10" s="90"/>
-      <c r="W10" s="121"/>
+      <c r="W10" s="112"/>
       <c r="Y10" s="79"/>
       <c r="Z10" s="79"/>
       <c r="AA10" s="79"/>
     </row>
     <row r="11" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="135">
+      <c r="B11" s="126">
         <f t="shared" ref="B11:B39" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="130" t="s">
+      <c r="C11" s="121" t="s">
         <v>162</v>
       </c>
       <c r="D11" s="43" t="s">
@@ -2496,18 +2496,18 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="V11" s="43"/>
-      <c r="W11" s="122"/>
+      <c r="W11" s="113"/>
       <c r="Y11" s="79"/>
       <c r="Z11" s="79"/>
       <c r="AA11" s="79"/>
     </row>
     <row r="12" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="135">
+      <c r="B12" s="126">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="131" t="s">
+      <c r="C12" s="122" t="s">
         <v>162</v>
       </c>
       <c r="D12" s="41" t="s">
@@ -2569,18 +2569,18 @@
         <v>1.764</v>
       </c>
       <c r="V12" s="41"/>
-      <c r="W12" s="123"/>
+      <c r="W12" s="114"/>
       <c r="Y12" s="79"/>
       <c r="Z12" s="79"/>
       <c r="AA12" s="79"/>
     </row>
     <row r="13" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="135">
+      <c r="B13" s="126">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="130" t="s">
+      <c r="C13" s="121" t="s">
         <v>162</v>
       </c>
       <c r="D13" s="43" t="s">
@@ -2642,18 +2642,18 @@
         <v>0.22</v>
       </c>
       <c r="V13" s="43"/>
-      <c r="W13" s="122"/>
+      <c r="W13" s="113"/>
       <c r="Y13" s="79"/>
       <c r="Z13" s="79"/>
       <c r="AA13" s="79"/>
     </row>
     <row r="14" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
-      <c r="B14" s="135">
+      <c r="B14" s="126">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="131" t="s">
+      <c r="C14" s="122" t="s">
         <v>162</v>
       </c>
       <c r="D14" s="41" t="s">
@@ -2715,18 +2715,18 @@
         <v>4.0619999999999994</v>
       </c>
       <c r="V14" s="41"/>
-      <c r="W14" s="124"/>
+      <c r="W14" s="115"/>
       <c r="Y14" s="79"/>
       <c r="Z14" s="79"/>
       <c r="AA14" s="79"/>
     </row>
     <row r="15" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="135">
+      <c r="B15" s="126">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="130" t="s">
+      <c r="C15" s="121" t="s">
         <v>162</v>
       </c>
       <c r="D15" s="43" t="s">
@@ -2788,18 +2788,18 @@
         <v>0.26</v>
       </c>
       <c r="V15" s="43"/>
-      <c r="W15" s="122"/>
+      <c r="W15" s="113"/>
       <c r="Y15" s="79"/>
       <c r="Z15" s="79"/>
       <c r="AA15" s="79"/>
     </row>
     <row r="16" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="135">
+      <c r="B16" s="126">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="131" t="s">
+      <c r="C16" s="122" t="s">
         <v>162</v>
       </c>
       <c r="D16" s="41" t="s">
@@ -2861,18 +2861,18 @@
         <v>29.534399999999998</v>
       </c>
       <c r="V16" s="41"/>
-      <c r="W16" s="124"/>
+      <c r="W16" s="115"/>
       <c r="Y16" s="79"/>
       <c r="Z16" s="79"/>
       <c r="AA16" s="79"/>
     </row>
     <row r="17" spans="1:27" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="136">
+      <c r="B17" s="127">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="132" t="s">
+      <c r="C17" s="123" t="s">
         <v>162</v>
       </c>
       <c r="D17" s="80" t="s">
@@ -2934,17 +2934,17 @@
         <v>9.6684000000000001</v>
       </c>
       <c r="V17" s="80"/>
-      <c r="W17" s="122"/>
+      <c r="W17" s="113"/>
       <c r="Y17" s="79"/>
       <c r="Z17" s="79"/>
     </row>
     <row r="18" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="135">
+      <c r="B18" s="126">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="131" t="s">
+      <c r="C18" s="122" t="s">
         <v>163</v>
       </c>
       <c r="D18" s="41" t="s">
@@ -3006,18 +3006,18 @@
         <v>1.548</v>
       </c>
       <c r="V18" s="41"/>
-      <c r="W18" s="123"/>
+      <c r="W18" s="114"/>
       <c r="Y18" s="79"/>
       <c r="Z18" s="79"/>
       <c r="AA18" s="79"/>
     </row>
     <row r="19" spans="1:27" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="135">
+      <c r="B19" s="126">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="130" t="s">
+      <c r="C19" s="121" t="s">
         <v>163</v>
       </c>
       <c r="D19" s="43" t="s">
@@ -3079,18 +3079,18 @@
         <v>1.252</v>
       </c>
       <c r="V19" s="43"/>
-      <c r="W19" s="122"/>
+      <c r="W19" s="113"/>
       <c r="Y19" s="79"/>
       <c r="Z19" s="79"/>
       <c r="AA19" s="79"/>
     </row>
     <row r="20" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
-      <c r="B20" s="135">
+      <c r="B20" s="126">
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
-      <c r="C20" s="131" t="s">
+      <c r="C20" s="122" t="s">
         <v>164</v>
       </c>
       <c r="D20" s="41" t="s">
@@ -3152,7 +3152,7 @@
         <v>9.0635999999999992</v>
       </c>
       <c r="V20" s="41"/>
-      <c r="W20" s="125" t="s">
+      <c r="W20" s="116" t="s">
         <v>214</v>
       </c>
       <c r="Y20" s="79"/>
@@ -3161,11 +3161,11 @@
     </row>
     <row r="21" spans="1:27" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
-      <c r="B21" s="135">
+      <c r="B21" s="126">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="130" t="s">
+      <c r="C21" s="121" t="s">
         <v>164</v>
       </c>
       <c r="D21" s="43" t="s">
@@ -3227,18 +3227,18 @@
         <v>3.5579999999999998</v>
       </c>
       <c r="V21" s="43"/>
-      <c r="W21" s="122"/>
+      <c r="W21" s="113"/>
       <c r="Y21" s="79"/>
       <c r="Z21" s="79"/>
       <c r="AA21" s="79"/>
     </row>
     <row r="22" spans="1:27" ht="25.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
-      <c r="B22" s="135">
+      <c r="B22" s="126">
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
-      <c r="C22" s="131" t="s">
+      <c r="C22" s="122" t="s">
         <v>164</v>
       </c>
       <c r="D22" s="41" t="s">
@@ -3300,7 +3300,7 @@
         <v>6.5190000000000001</v>
       </c>
       <c r="V22" s="41"/>
-      <c r="W22" s="126" t="s">
+      <c r="W22" s="117" t="s">
         <v>215</v>
       </c>
       <c r="Y22" s="79"/>
@@ -3309,11 +3309,11 @@
     </row>
     <row r="23" spans="1:27" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
-      <c r="B23" s="135">
+      <c r="B23" s="126">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="130" t="s">
+      <c r="C23" s="121" t="s">
         <v>165</v>
       </c>
       <c r="D23" s="43" t="s">
@@ -3375,18 +3375,18 @@
         <v>10.693200000000001</v>
       </c>
       <c r="V23" s="43"/>
-      <c r="W23" s="122"/>
+      <c r="W23" s="113"/>
       <c r="Y23" s="79"/>
       <c r="Z23" s="79"/>
       <c r="AA23" s="79"/>
     </row>
     <row r="24" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
-      <c r="B24" s="135">
+      <c r="B24" s="126">
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
-      <c r="C24" s="131" t="s">
+      <c r="C24" s="122" t="s">
         <v>166</v>
       </c>
       <c r="D24" s="41" t="s">
@@ -3448,18 +3448,18 @@
         <v>0.755</v>
       </c>
       <c r="V24" s="41"/>
-      <c r="W24" s="123"/>
+      <c r="W24" s="114"/>
       <c r="Y24" s="79"/>
       <c r="Z24" s="79"/>
       <c r="AA24" s="79"/>
     </row>
     <row r="25" spans="1:27" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
-      <c r="B25" s="135">
+      <c r="B25" s="126">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="130" t="s">
+      <c r="C25" s="121" t="s">
         <v>167</v>
       </c>
       <c r="D25" s="43" t="s">
@@ -3523,18 +3523,18 @@
       <c r="V25" s="43" t="s">
         <v>215</v>
       </c>
-      <c r="W25" s="122"/>
+      <c r="W25" s="113"/>
       <c r="Y25" s="79"/>
       <c r="Z25" s="79"/>
       <c r="AA25" s="79"/>
     </row>
     <row r="26" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
-      <c r="B26" s="135">
+      <c r="B26" s="126">
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
-      <c r="C26" s="131" t="s">
+      <c r="C26" s="122" t="s">
         <v>168</v>
       </c>
       <c r="D26" s="41" t="s">
@@ -3596,18 +3596,18 @@
         <v>4.47</v>
       </c>
       <c r="V26" s="46"/>
-      <c r="W26" s="123"/>
+      <c r="W26" s="114"/>
       <c r="Y26" s="79"/>
       <c r="Z26" s="79"/>
       <c r="AA26" s="79"/>
     </row>
     <row r="27" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
-      <c r="B27" s="135">
+      <c r="B27" s="126">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="130" t="s">
+      <c r="C27" s="121" t="s">
         <v>168</v>
       </c>
       <c r="D27" s="43" t="s">
@@ -3669,18 +3669,18 @@
         <v>0.76500000000000001</v>
       </c>
       <c r="V27" s="43"/>
-      <c r="W27" s="122"/>
+      <c r="W27" s="113"/>
       <c r="Y27" s="79"/>
       <c r="Z27" s="79"/>
       <c r="AA27" s="79"/>
     </row>
     <row r="28" spans="1:27" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
-      <c r="B28" s="135">
+      <c r="B28" s="126">
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
-      <c r="C28" s="131" t="s">
+      <c r="C28" s="122" t="s">
         <v>168</v>
       </c>
       <c r="D28" s="41" t="s">
@@ -3742,18 +3742,18 @@
         <v>0.42</v>
       </c>
       <c r="V28" s="41"/>
-      <c r="W28" s="123"/>
+      <c r="W28" s="114"/>
       <c r="Y28" s="79"/>
       <c r="Z28" s="79"/>
       <c r="AA28" s="79"/>
     </row>
     <row r="29" spans="1:27" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
-      <c r="B29" s="135">
+      <c r="B29" s="126">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="130" t="s">
+      <c r="C29" s="121" t="s">
         <v>168</v>
       </c>
       <c r="D29" s="43" t="s">
@@ -3815,18 +3815,18 @@
         <v>0.44</v>
       </c>
       <c r="V29" s="43"/>
-      <c r="W29" s="122"/>
+      <c r="W29" s="113"/>
       <c r="Y29" s="79"/>
       <c r="Z29" s="79"/>
       <c r="AA29" s="79"/>
     </row>
     <row r="30" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
-      <c r="B30" s="135">
+      <c r="B30" s="126">
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
-      <c r="C30" s="131" t="s">
+      <c r="C30" s="122" t="s">
         <v>168</v>
       </c>
       <c r="D30" s="41" t="s">
@@ -3888,18 +3888,18 @@
         <v>0.13</v>
       </c>
       <c r="V30" s="41"/>
-      <c r="W30" s="123"/>
+      <c r="W30" s="114"/>
       <c r="Y30" s="79"/>
       <c r="Z30" s="79"/>
       <c r="AA30" s="79"/>
     </row>
     <row r="31" spans="1:27" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
-      <c r="B31" s="135">
+      <c r="B31" s="126">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C31" s="130" t="s">
+      <c r="C31" s="121" t="s">
         <v>168</v>
       </c>
       <c r="D31" s="43" t="s">
@@ -3961,18 +3961,18 @@
         <v>0.20500000000000002</v>
       </c>
       <c r="V31" s="43"/>
-      <c r="W31" s="122"/>
+      <c r="W31" s="113"/>
       <c r="Y31" s="79"/>
       <c r="Z31" s="79"/>
       <c r="AA31" s="79"/>
     </row>
     <row r="32" spans="1:27" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
-      <c r="B32" s="135">
+      <c r="B32" s="126">
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="131" t="s">
+      <c r="C32" s="122" t="s">
         <v>168</v>
       </c>
       <c r="D32" s="41" t="s">
@@ -4034,18 +4034,18 @@
         <v>3.7744</v>
       </c>
       <c r="V32" s="41"/>
-      <c r="W32" s="123"/>
+      <c r="W32" s="114"/>
       <c r="Y32" s="79"/>
       <c r="Z32" s="79"/>
       <c r="AA32" s="79"/>
     </row>
     <row r="33" spans="1:31" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
-      <c r="B33" s="135">
+      <c r="B33" s="126">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="130" t="s">
+      <c r="C33" s="121" t="s">
         <v>168</v>
       </c>
       <c r="D33" s="43" t="s">
@@ -4107,7 +4107,7 @@
         <v>0.1</v>
       </c>
       <c r="V33" s="43"/>
-      <c r="W33" s="122"/>
+      <c r="W33" s="113"/>
       <c r="X33" s="79"/>
       <c r="Y33" s="79"/>
       <c r="Z33" s="79"/>
@@ -4119,11 +4119,11 @@
     </row>
     <row r="34" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
-      <c r="B34" s="135">
+      <c r="B34" s="126">
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="133" t="s">
+      <c r="C34" s="124" t="s">
         <v>183</v>
       </c>
       <c r="D34" s="44" t="s">
@@ -4185,7 +4185,7 @@
       <c r="V34" s="44" t="s">
         <v>185</v>
       </c>
-      <c r="W34" s="127"/>
+      <c r="W34" s="118"/>
       <c r="X34" s="79"/>
       <c r="Y34" s="79"/>
       <c r="Z34" s="79"/>
@@ -4197,11 +4197,11 @@
     </row>
     <row r="35" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
-      <c r="B35" s="135">
+      <c r="B35" s="126">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="130" t="s">
+      <c r="C35" s="121" t="s">
         <v>171</v>
       </c>
       <c r="D35" s="43" t="s">
@@ -4263,7 +4263,7 @@
         <v>12.0036</v>
       </c>
       <c r="V35" s="43"/>
-      <c r="W35" s="122"/>
+      <c r="W35" s="113"/>
       <c r="X35" s="79"/>
       <c r="Y35" s="79"/>
       <c r="Z35" s="79"/>
@@ -4275,11 +4275,11 @@
     </row>
     <row r="36" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
-      <c r="B36" s="135">
+      <c r="B36" s="126">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="131" t="s">
+      <c r="C36" s="122" t="s">
         <v>170</v>
       </c>
       <c r="D36" s="41" t="s">
@@ -4341,7 +4341,7 @@
         <v>243.99629999999999</v>
       </c>
       <c r="V36" s="41"/>
-      <c r="W36" s="123"/>
+      <c r="W36" s="114"/>
       <c r="X36" s="79"/>
       <c r="Y36" s="79"/>
       <c r="Z36" s="79"/>
@@ -4353,11 +4353,11 @@
     </row>
     <row r="37" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
-      <c r="B37" s="135">
+      <c r="B37" s="126">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C37" s="130" t="s">
+      <c r="C37" s="121" t="s">
         <v>170</v>
       </c>
       <c r="D37" s="43" t="s">
@@ -4419,7 +4419,7 @@
         <v>14.825700000000001</v>
       </c>
       <c r="V37" s="43"/>
-      <c r="W37" s="122"/>
+      <c r="W37" s="113"/>
       <c r="X37" s="79"/>
       <c r="Y37" s="79"/>
       <c r="Z37" s="79"/>
@@ -4431,11 +4431,11 @@
     </row>
     <row r="38" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
-      <c r="B38" s="135">
+      <c r="B38" s="126">
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
-      <c r="C38" s="131" t="s">
+      <c r="C38" s="122" t="s">
         <v>170</v>
       </c>
       <c r="D38" s="41" t="s">
@@ -4497,18 +4497,18 @@
         <v>8.7399000000000004</v>
       </c>
       <c r="V38" s="41"/>
-      <c r="W38" s="123"/>
+      <c r="W38" s="114"/>
       <c r="Y38" s="79"/>
       <c r="Z38" s="79"/>
       <c r="AA38" s="79"/>
     </row>
     <row r="39" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
-      <c r="B39" s="135">
+      <c r="B39" s="126">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C39" s="130" t="s">
+      <c r="C39" s="121" t="s">
         <v>166</v>
       </c>
       <c r="D39" s="43" t="s">
@@ -4570,18 +4570,18 @@
         <v>8.2080000000000002</v>
       </c>
       <c r="V39" s="43"/>
-      <c r="W39" s="122"/>
+      <c r="W39" s="113"/>
       <c r="Y39" s="79"/>
       <c r="Z39" s="79"/>
       <c r="AA39" s="79"/>
     </row>
     <row r="40" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
-      <c r="B40" s="135">
+      <c r="B40" s="126">
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
-      <c r="C40" s="134" t="s">
+      <c r="C40" s="125" t="s">
         <v>169</v>
       </c>
       <c r="D40" s="50" t="s">
@@ -4645,7 +4645,7 @@
       <c r="V40" s="89" t="s">
         <v>214</v>
       </c>
-      <c r="W40" s="128"/>
+      <c r="W40" s="119"/>
       <c r="Y40" s="79"/>
       <c r="Z40" s="79"/>
       <c r="AA40" s="79"/>
@@ -4667,10 +4667,10 @@
       <c r="N41" s="28"/>
       <c r="O41" s="28"/>
       <c r="P41" s="28"/>
-      <c r="Q41" s="106" t="s">
+      <c r="Q41" s="133" t="s">
         <v>186</v>
       </c>
-      <c r="R41" s="107"/>
+      <c r="R41" s="134"/>
       <c r="S41" s="99">
         <f>SUM(S10:S40)</f>
         <v>177.0273</v>
@@ -4702,10 +4702,10 @@
       <c r="N42" s="7"/>
       <c r="O42" s="7"/>
       <c r="P42" s="7"/>
-      <c r="Q42" s="108" t="s">
+      <c r="Q42" s="135" t="s">
         <v>187</v>
       </c>
-      <c r="R42" s="109"/>
+      <c r="R42" s="136"/>
       <c r="S42" s="100">
         <f>S41/10</f>
         <v>17.702729999999999</v>

</xml_diff>